<commit_message>
Rename dashboard title to Stock Report HQ
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/10-2/Stock Daily 2026-10-02.xlsx
+++ b/10-2/Stock Daily 2026-10-02.xlsx
@@ -4266,11 +4266,11 @@
         </is>
       </c>
       <c r="C31" s="206" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D31" s="207" t="n"/>
       <c r="E31" s="207" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F31" s="207" t="n"/>
       <c r="G31" s="207" t="n"/>

</xml_diff>